<commit_message>
Update images, BOMs and MM-BASE firmware
</commit_message>
<xml_diff>
--- a/modules/mm-air/bom/mm-air-gen1-reva-bom.xlsx
+++ b/modules/mm-air/bom/mm-air-gen1-reva-bom.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andre\Desktop\MakaniMotion\Engineering\mm-fan-gen1\mm-fan-gen1\modules\mm-air\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2040944E-F024-47FA-BDA6-E834169497F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA1200DD-4BAC-450D-ABA9-530B9A900599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" xr2:uid="{790FE4A5-72AF-4AEE-9175-50CBEDA28C41}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{790FE4A5-72AF-4AEE-9175-50CBEDA28C41}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -156,9 +156,6 @@
     <t>Screw M3 x 30mm</t>
   </si>
   <si>
-    <t>Screw M3 x 5mm</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
@@ -190,6 +187,9 @@
   </si>
   <si>
     <t>mm-air-shroud-gen1-reva</t>
+  </si>
+  <si>
+    <t>Screw M3 x 6mm</t>
   </si>
 </sst>
 </file>
@@ -722,7 +722,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="30">
+    <row r="7" spans="1:14">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -733,7 +733,7 @@
         <v>5</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>6</v>
@@ -773,7 +773,7 @@
         <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -859,7 +859,7 @@
         <v>33</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E13">
         <v>4</v>
@@ -873,10 +873,10 @@
         <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E14">
         <v>2</v>
@@ -893,7 +893,7 @@
         <v>32</v>
       </c>
       <c r="D15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E15">
         <v>4</v>
@@ -907,10 +907,10 @@
         <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -919,10 +919,10 @@
         <v>16</v>
       </c>
       <c r="G16" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16" s="8" t="s">
         <v>43</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -930,10 +930,10 @@
         <v>7</v>
       </c>
       <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" t="s">
         <v>40</v>
-      </c>
-      <c r="D17" t="s">
-        <v>41</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -942,10 +942,10 @@
         <v>16</v>
       </c>
       <c r="G17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -953,7 +953,7 @@
         <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E18">
         <v>1</v>

</xml_diff>